<commit_message>
在 vscode 的專案設定檔：　.vscode\settings.json 設定 python.defaultIntepert 。
</commit_message>
<xml_diff>
--- a/output7/【河洛文讀注音-注音二式】《詩經．小雅．鹿鳴》.xlsx
+++ b/output7/【河洛文讀注音-注音二式】《詩經．小雅．鹿鳴》.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Piau-Im\output7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{103C102B-9689-4ED8-A9C4-0E93E031541B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C29F13C-AD23-4BE0-86EB-4DB5C5321161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="195" yWindow="2595" windowWidth="28800" windowHeight="11295" activeTab="4" xr2:uid="{25A76161-EFED-4AC8-8EAA-A42737AE1909}"/>
+    <workbookView xWindow="105" yWindow="2595" windowWidth="28695" windowHeight="11295" activeTab="4" xr2:uid="{25A76161-EFED-4AC8-8EAA-A42737AE1909}"/>
   </bookViews>
   <sheets>
     <sheet name="env" sheetId="8" r:id="rId1"/>

</xml_diff>